<commit_message>
ios 1.2: app per Apple Watch (schermata, complicazioni, impostazioni dal telefono)
Target StepTellerWatch e StepTellerWatchWidgets in project.yml (watchOS 10+, incorporati nell'app iPhone).
Una schermata in stile «Dan Dan Dan» (palette notte) con serie, Jolly, passi di oggi letti da Salute
sull'orologio, obiettivo, barra e minuti che mancano; complicazioni tondo, rettangolo, riga e angolo
con il codice del blocco schermo. Obiettivo, velocità, unità, serie, Jolly e taratura arrivano dal
telefono con WatchConnectivity (WatchPayload/WatchSync) e restano sull'orologio. Nucleo compilato anche
per watchOS. Testi nuovi in 10 lingue (bozze), cataloghi per i permessi del Watch, registro 1.2 aperto
in parallelo alla 1.1 (caso particolare in RILASCIO.md), CI senza -sdk iphonesimulator.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ios/localizzazione/NEAT_testi_tradotti.xlsx
+++ b/ios/localizzazione/NEAT_testi_tradotti.xlsx
@@ -1473,7 +1473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P203"/>
+  <dimension ref="A1:P207"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -18120,6 +18120,334 @@
         </is>
       </c>
     </row>
+    <row r="204">
+      <c r="A204" s="5" t="inlineStr">
+        <is>
+          <t>w.watch.gallery.desc</t>
+        </is>
+      </c>
+      <c r="B204" s="5" t="inlineStr">
+        <is>
+          <t>Apple Watch</t>
+        </is>
+      </c>
+      <c r="C204" s="5" t="inlineStr">
+        <is>
+          <t>Sistema</t>
+        </is>
+      </c>
+      <c r="D204" s="5" t="inlineStr">
+        <is>
+          <t>Descrizione delle complicazioni nella scelta del quadrante dell'Apple Watch (al posto di w.gallery.desc, che parla del blocco schermo).</t>
+        </is>
+      </c>
+      <c r="E204" s="5" t="inlineStr">
+        <is>
+          <t>≤ 70</t>
+        </is>
+      </c>
+      <c r="F204" s="7" t="inlineStr">
+        <is>
+          <t>Passi, minuti che mancano e serie, sul quadrante.</t>
+        </is>
+      </c>
+      <c r="G204" s="6" t="inlineStr">
+        <is>
+          <t>Steps, minutes left and your streak, right on your watch face.</t>
+        </is>
+      </c>
+      <c r="H204" s="6" t="inlineStr">
+        <is>
+          <t>Pasos, minutos restantes y racha, en la esfera del reloj.</t>
+        </is>
+      </c>
+      <c r="I204" s="6" t="inlineStr">
+        <is>
+          <t>Pas, minutes restantes et série, sur le cadran.</t>
+        </is>
+      </c>
+      <c r="J204" s="6" t="inlineStr">
+        <is>
+          <t>Schritte, übrige Minuten und Serie, direkt auf dem Zifferblatt.</t>
+        </is>
+      </c>
+      <c r="K204" s="6" t="inlineStr">
+        <is>
+          <t>Passos, minutos restantes e sequência, no mostrador do relógio.</t>
+        </is>
+      </c>
+      <c r="L204" s="6" t="inlineStr">
+        <is>
+          <t>歩数、残り時間、連続記録を文字盤でチェック。</t>
+        </is>
+      </c>
+      <c r="M204" s="6" t="inlineStr">
+        <is>
+          <t>시계 페이스에서 걸음 수, 남은 시간, 연속 기록을 확인해요.</t>
+        </is>
+      </c>
+      <c r="N204" s="6" t="inlineStr">
+        <is>
+          <t>步数、剩余分钟数和连续记录，表盘上就能看。</t>
+        </is>
+      </c>
+      <c r="O204" s="6" t="inlineStr">
+        <is>
+          <t>步數、剩餘分鐘數和連續紀錄，錶面上就能看。</t>
+        </is>
+      </c>
+      <c r="P204" s="6" t="inlineStr">
+        <is>
+          <t>Bozza di Claude (1.2), da confermare con ChatGPT.</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="5" t="inlineStr">
+        <is>
+          <t>w.watch.nodata</t>
+        </is>
+      </c>
+      <c r="B205" s="5" t="inlineStr">
+        <is>
+          <t>Apple Watch</t>
+        </is>
+      </c>
+      <c r="C205" s="5" t="inlineStr">
+        <is>
+          <t>Visibile</t>
+        </is>
+      </c>
+      <c r="D205" s="5" t="inlineStr">
+        <is>
+          <t>App per Apple Watch: riga sotto la barra quando Salute non dà passi (permesso negato o nessun dato), al posto dei minuti che mancano, MAIUSCOLO.</t>
+        </is>
+      </c>
+      <c r="E205" s="5" t="inlineStr">
+        <is>
+          <t>≤ 22</t>
+        </is>
+      </c>
+      <c r="F205" s="7" t="inlineStr">
+        <is>
+          <t>NIENTE DATI DA SALUTE</t>
+        </is>
+      </c>
+      <c r="G205" s="6" t="inlineStr">
+        <is>
+          <t>NO HEALTH DATA</t>
+        </is>
+      </c>
+      <c r="H205" s="6" t="inlineStr">
+        <is>
+          <t>SIN DATOS DE SALUD</t>
+        </is>
+      </c>
+      <c r="I205" s="6" t="inlineStr">
+        <is>
+          <t>PAS DE DONNÉES SANTÉ</t>
+        </is>
+      </c>
+      <c r="J205" s="6" t="inlineStr">
+        <is>
+          <t>KEINE HEALTH-DATEN</t>
+        </is>
+      </c>
+      <c r="K205" s="6" t="inlineStr">
+        <is>
+          <t>SEM DADOS DO SAÚDE</t>
+        </is>
+      </c>
+      <c r="L205" s="6" t="inlineStr">
+        <is>
+          <t>ヘルスケアのデータなし</t>
+        </is>
+      </c>
+      <c r="M205" s="6" t="inlineStr">
+        <is>
+          <t>건강 데이터 없음</t>
+        </is>
+      </c>
+      <c r="N205" s="6" t="inlineStr">
+        <is>
+          <t>无“健康”数据</t>
+        </is>
+      </c>
+      <c r="O205" s="6" t="inlineStr">
+        <is>
+          <t>無「健康」資料</t>
+        </is>
+      </c>
+      <c r="P205" s="6" t="inlineStr">
+        <is>
+          <t>Bozza di Claude (1.2), da confermare con ChatGPT.</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="5" t="inlineStr">
+        <is>
+          <t>w.watch.nodata.vo</t>
+        </is>
+      </c>
+      <c r="B206" s="5" t="inlineStr">
+        <is>
+          <t>Apple Watch</t>
+        </is>
+      </c>
+      <c r="C206" s="5" t="inlineStr">
+        <is>
+          <t>VoiceOver</t>
+        </is>
+      </c>
+      <c r="D206" s="5" t="inlineStr">
+        <is>
+          <t>Descrizione letta ad alta voce nello stesso caso: dice dove controllare il permesso.</t>
+        </is>
+      </c>
+      <c r="E206" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F206" s="7" t="inlineStr">
+        <is>
+          <t>Nessun dato da Salute. Controlla i permessi di NEAT nell'app Salute del telefono.</t>
+        </is>
+      </c>
+      <c r="G206" s="6" t="inlineStr">
+        <is>
+          <t>No data from Health. Check NEAT's permissions in the Health app on your iPhone.</t>
+        </is>
+      </c>
+      <c r="H206" s="6" t="inlineStr">
+        <is>
+          <t>No hay datos de Salud. Revisa los permisos de NEAT en la app Salud del iPhone.</t>
+        </is>
+      </c>
+      <c r="I206" s="6" t="inlineStr">
+        <is>
+          <t>Aucune donnée de Santé. Vérifie les autorisations de NEAT dans l’app Santé de l’iPhone.</t>
+        </is>
+      </c>
+      <c r="J206" s="6" t="inlineStr">
+        <is>
+          <t>Keine Daten aus Health. Prüfe die Berechtigungen von NEAT in der Health-App auf dem iPhone.</t>
+        </is>
+      </c>
+      <c r="K206" s="6" t="inlineStr">
+        <is>
+          <t>Sem dados do Saúde. Verifique as permissões do NEAT no app Saúde do iPhone.</t>
+        </is>
+      </c>
+      <c r="L206" s="6" t="inlineStr">
+        <is>
+          <t>ヘルスケアのデータがありません。iPhoneのヘルスケアアプリでNEATのアクセス権を確認してください。</t>
+        </is>
+      </c>
+      <c r="M206" s="6" t="inlineStr">
+        <is>
+          <t>건강 앱 데이터가 없어요. iPhone의 건강 앱에서 NEAT의 권한을 확인해 주세요.</t>
+        </is>
+      </c>
+      <c r="N206" s="6" t="inlineStr">
+        <is>
+          <t>没有来自“健康”的数据。请在 iPhone 的“健康”App 中检查 NEAT 的权限。</t>
+        </is>
+      </c>
+      <c r="O206" s="6" t="inlineStr">
+        <is>
+          <t>沒有來自「健康」的資料。請在 iPhone 的「健康」App 中檢查 NEAT 的權限。</t>
+        </is>
+      </c>
+      <c r="P206" s="6" t="inlineStr">
+        <is>
+          <t>Bozza di Claude (1.2), da confermare con ChatGPT.</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="5" t="inlineStr">
+        <is>
+          <t>p.health.watch</t>
+        </is>
+      </c>
+      <c r="B207" s="5" t="inlineStr">
+        <is>
+          <t>Permessi (finestre di watchOS)</t>
+        </is>
+      </c>
+      <c r="C207" s="5" t="inlineStr">
+        <is>
+          <t>Sistema</t>
+        </is>
+      </c>
+      <c r="D207" s="5" t="inlineStr">
+        <is>
+          <t>Testo mostrato quando l'app per Apple Watch chiede di leggere i passi da Salute. Tono formale-chiaro, controllato da Apple.</t>
+        </is>
+      </c>
+      <c r="E207" s="5" t="inlineStr">
+        <is>
+          <t>≤ 200</t>
+        </is>
+      </c>
+      <c r="F207" s="7" t="inlineStr">
+        <is>
+          <t>NEAT legge i tuoi passi di oggi da Salute per mostrarli sull'orologio e stimare i minuti che mancano. Non scrive nulla e non invia dati fuori dall'orologio.</t>
+        </is>
+      </c>
+      <c r="G207" s="6" t="inlineStr">
+        <is>
+          <t>NEAT reads today's steps from Health to show them on your watch and estimate the minutes left. It writes nothing and sends no data off your watch.</t>
+        </is>
+      </c>
+      <c r="H207" s="6" t="inlineStr">
+        <is>
+          <t>NEAT lee tus pasos de hoy de Salud para mostrarlos en el reloj y estimar los minutos que faltan. No escribe nada ni envía datos fuera del reloj.</t>
+        </is>
+      </c>
+      <c r="I207" s="6" t="inlineStr">
+        <is>
+          <t>NEAT lit tes pas du jour dans Santé pour les afficher sur la montre et estimer les minutes restantes. Aucune écriture ni envoi de données hors de la montre.</t>
+        </is>
+      </c>
+      <c r="J207" s="6" t="inlineStr">
+        <is>
+          <t>NEAT liest heutige Schritte aus Health, um sie auf der Uhr anzuzeigen und die übrigen Minuten zu schätzen. Schreibt nichts und sendet keine Daten von der Uhr.</t>
+        </is>
+      </c>
+      <c r="K207" s="6" t="inlineStr">
+        <is>
+          <t>O NEAT lê seus passos de hoje no Saúde para mostrá-los no relógio e estimar os minutos restantes. Não grava nada nem envia dados para fora do relógio.</t>
+        </is>
+      </c>
+      <c r="L207" s="6" t="inlineStr">
+        <is>
+          <t>NEATはヘルスケアから今日の歩数を読み取ってApple Watchに表示し、残りの時間を推定します。データの書き込みや外部への送信は行いません。</t>
+        </is>
+      </c>
+      <c r="M207" s="6" t="inlineStr">
+        <is>
+          <t>NEAT는 건강 앱에서 오늘 걸음 수를 읽어 시계에 표시하고 남은 시간을 추정합니다. 데이터를 쓰거나 시계 밖으로 보내지 않습니다.</t>
+        </is>
+      </c>
+      <c r="N207" s="6" t="inlineStr">
+        <is>
+          <t>NEAT从“健康”读取今日步数，在手表上显示并估算剩余分钟数。不写入任何内容，也不向手表外发送数据。</t>
+        </is>
+      </c>
+      <c r="O207" s="6" t="inlineStr">
+        <is>
+          <t>NEAT從「健康」讀取今日步數，在手錶上顯示並估算剩餘分鐘數。不寫入任何內容，也不向手錶外傳送資料。</t>
+        </is>
+      </c>
+      <c r="P207" s="6" t="inlineStr">
+        <is>
+          <t>Bozza di Claude (1.2), da confermare con ChatGPT.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:P192"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>